<commit_message>
Add feature tests for attendance reporting and student enrollment
</commit_message>
<xml_diff>
--- a/resources/templates/students-template.xlsx
+++ b/resources/templates/students-template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
   <si>
     <t>student_number</t>
   </si>
@@ -54,9 +54,6 @@
   </si>
   <si>
     <t>appreciation_score</t>
-  </si>
-  <si>
-    <t>absences_count</t>
   </si>
   <si>
     <t>appreciation</t>
@@ -377,18 +374,18 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="8.59765625" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="11.06" customWidth="true" style="0"/>
     <col min="3" max="3" width="10.58" customWidth="true" style="0"/>
     <col min="4" max="4" width="11.55" customWidth="true" style="0"/>
     <col min="13" max="13" width="10.16" customWidth="true" style="0"/>
-    <col min="19" max="19" width="19.86" customWidth="true" style="0"/>
-    <col min="21" max="21" width="13" customWidth="true" style="0"/>
+    <col min="18" max="18" width="19.86" customWidth="true" style="0"/>
+    <col min="20" max="20" width="13" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" customHeight="1" ht="46.25" s="3" customFormat="1">
+    <row r="1" spans="1:20" customHeight="1" ht="46.25" s="3" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -431,15 +428,12 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>